<commit_message>
data: actualizar 16 fichas a version HISMINSA 25/05/2026
</commit_message>
<xml_diff>
--- a/data/Ficha_04_DL1153_202605_Menor_02años_Crecimiento_Inadecuado.xlsx
+++ b/data/Ficha_04_DL1153_202605_Menor_02años_Crecimiento_Inadecuado.xlsx
@@ -958,7 +958,7 @@
     <t>PERIODO: ENERO - MAYO 2026</t>
   </si>
   <si>
-    <t>FUENTE: HISMINSA: 17/05/2026</t>
+    <t>FUENTE: HISMINSA: 24/05/2026</t>
   </si>
 </sst>
 </file>
@@ -1469,7 +1469,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1" refreshedBy="TuSoft" refreshedDate="46160.518211342591" createdVersion="6" refreshedVersion="6" minRefreshableVersion="3" recordCount="188">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1" refreshedBy="TuSoft" refreshedDate="46167.519208796293" createdVersion="6" refreshedVersion="6" minRefreshableVersion="3" recordCount="188">
   <cacheSource type="worksheet">
     <worksheetSource name="Tabla1"/>
   </cacheSource>
@@ -1601,7 +1601,7 @@
       <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="0" maxValue="1"/>
     </cacheField>
     <cacheField name="fecha_num1" numFmtId="14">
-      <sharedItems containsNonDate="0" containsDate="1" containsString="0" containsBlank="1" minDate="2026-01-01T00:00:00" maxDate="2026-05-14T00:00:00"/>
+      <sharedItems containsNonDate="0" containsDate="1" containsString="0" containsBlank="1" minDate="2026-01-01T00:00:00" maxDate="2026-05-20T00:00:00"/>
     </cacheField>
     <cacheField name="num_2" numFmtId="0">
       <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="0" maxValue="0"/>
@@ -4450,9 +4450,9 @@
     <s v="94490596"/>
     <d v="2026-01-29T00:00:00"/>
     <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <m/>
+    <n v="1"/>
+    <n v="1"/>
+    <d v="2026-05-02T00:00:00"/>
     <n v="0"/>
     <m/>
   </r>
@@ -4479,7 +4479,7 @@
   </r>
   <r>
     <x v="0"/>
-    <x v="3"/>
+    <x v="0"/>
     <s v="HUANCAVELICA"/>
     <x v="0"/>
     <x v="26"/>
@@ -4490,11 +4490,11 @@
     <s v="SAN CRISTOBAL"/>
     <n v="3861"/>
     <s v="94241877"/>
-    <d v="2025-10-10T00:00:00"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <m/>
+    <d v="2026-02-12T00:00:00"/>
+    <n v="1"/>
+    <n v="1"/>
+    <n v="1"/>
+    <d v="2026-05-19T00:00:00"/>
     <n v="0"/>
     <m/>
   </r>
@@ -4660,9 +4660,9 @@
     <s v="94201689"/>
     <d v="2026-02-06T00:00:00"/>
     <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <m/>
+    <n v="1"/>
+    <n v="1"/>
+    <d v="2026-05-16T00:00:00"/>
     <n v="0"/>
     <m/>
   </r>
@@ -5573,129 +5573,6 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica7" cacheId="37" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
-  <location ref="J8:N14" firstHeaderRow="0" firstDataRow="1" firstDataCol="2" rowPageCount="1" colPageCount="1"/>
-  <pivotFields count="20">
-    <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
-      <items count="1">
-        <item x="0"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
-      <items count="5">
-        <item x="3"/>
-        <item x="2"/>
-        <item x="4"/>
-        <item x="1"/>
-        <item x="0"/>
-      </items>
-    </pivotField>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField axis="axisPage" compact="0" outline="0" showAll="0">
-      <items count="7">
-        <item x="1"/>
-        <item x="3"/>
-        <item x="2"/>
-        <item x="0"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" numFmtId="164" outline="0" showAll="0"/>
-    <pivotField dataField="1" compact="0" outline="0" showAll="0"/>
-    <pivotField dataField="1" compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField compact="0" outline="0" showAll="0"/>
-    <pivotField dataField="1" compact="0" outline="0" dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
-  </pivotFields>
-  <rowFields count="2">
-    <field x="0"/>
-    <field x="1"/>
-  </rowFields>
-  <rowItems count="6">
-    <i>
-      <x/>
-      <x/>
-    </i>
-    <i r="1">
-      <x v="1"/>
-    </i>
-    <i r="1">
-      <x v="2"/>
-    </i>
-    <i r="1">
-      <x v="3"/>
-    </i>
-    <i r="1">
-      <x v="4"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="-2"/>
-  </colFields>
-  <colItems count="3">
-    <i>
-      <x/>
-    </i>
-    <i i="1">
-      <x v="1"/>
-    </i>
-    <i i="2">
-      <x v="2"/>
-    </i>
-  </colItems>
-  <pageFields count="1">
-    <pageField fld="3" hier="-1"/>
-  </pageFields>
-  <dataFields count="3">
-    <dataField name="Suma de den" fld="13" baseField="0" baseItem="0"/>
-    <dataField name="Suma de num" fld="14" baseField="0" baseItem="0"/>
-    <dataField name="Suma de Indicador" fld="19" baseField="0" baseItem="0" numFmtId="165"/>
-  </dataFields>
-  <formats count="2">
-    <format dxfId="26">
-      <pivotArea outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="2"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-    <format dxfId="25">
-      <pivotArea outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="2"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </format>
-  </formats>
-  <pivotTableStyleInfo name="PivotStyleMedium13" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica6" cacheId="37" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
   <location ref="A8:G15" firstHeaderRow="0" firstDataRow="1" firstDataCol="4" rowPageCount="2" colPageCount="1"/>
   <pivotFields count="20">
@@ -5860,6 +5737,129 @@
   <pageFields count="2">
     <pageField fld="0" hier="-1"/>
     <pageField fld="1" hier="-1"/>
+  </pageFields>
+  <dataFields count="3">
+    <dataField name="Suma de den" fld="13" baseField="0" baseItem="0"/>
+    <dataField name="Suma de num" fld="14" baseField="0" baseItem="0"/>
+    <dataField name="Suma de Indicador" fld="19" baseField="0" baseItem="0" numFmtId="165"/>
+  </dataFields>
+  <formats count="2">
+    <format dxfId="26">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="25">
+      <pivotArea outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+  </formats>
+  <pivotTableStyleInfo name="PivotStyleMedium13" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="TablaDinámica7" cacheId="37" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="6" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="6" indent="0" compact="0" compactData="0" multipleFieldFilters="0">
+  <location ref="J8:N14" firstHeaderRow="0" firstDataRow="1" firstDataCol="2" rowPageCount="1" colPageCount="1"/>
+  <pivotFields count="20">
+    <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
+      <items count="1">
+        <item x="0"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
+      <items count="5">
+        <item x="3"/>
+        <item x="2"/>
+        <item x="4"/>
+        <item x="1"/>
+        <item x="0"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField axis="axisPage" compact="0" outline="0" showAll="0">
+      <items count="7">
+        <item x="1"/>
+        <item x="3"/>
+        <item x="2"/>
+        <item x="0"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" numFmtId="164" outline="0" showAll="0"/>
+    <pivotField dataField="1" compact="0" outline="0" showAll="0"/>
+    <pivotField dataField="1" compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField compact="0" outline="0" showAll="0"/>
+    <pivotField dataField="1" compact="0" outline="0" dragToRow="0" dragToCol="0" dragToPage="0" showAll="0" defaultSubtotal="0"/>
+  </pivotFields>
+  <rowFields count="2">
+    <field x="0"/>
+    <field x="1"/>
+  </rowFields>
+  <rowItems count="6">
+    <i>
+      <x/>
+      <x/>
+    </i>
+    <i r="1">
+      <x v="1"/>
+    </i>
+    <i r="1">
+      <x v="2"/>
+    </i>
+    <i r="1">
+      <x v="3"/>
+    </i>
+    <i r="1">
+      <x v="4"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="-2"/>
+  </colFields>
+  <colItems count="3">
+    <i>
+      <x/>
+    </i>
+    <i i="1">
+      <x v="1"/>
+    </i>
+    <i i="2">
+      <x v="2"/>
+    </i>
+  </colItems>
+  <pageFields count="1">
+    <pageField fld="3" hier="-1"/>
   </pageFields>
   <dataFields count="3">
     <dataField name="Suma de den" fld="13" baseField="0" baseItem="0"/>
@@ -6345,13 +6345,13 @@
         <v>1</v>
       </c>
       <c r="L9" s="4">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="M9" s="4">
         <v>8</v>
       </c>
       <c r="N9" s="5">
-        <v>0.15384615384615385</v>
+        <v>0.15686274509803921</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
@@ -6414,10 +6414,10 @@
         <v>150</v>
       </c>
       <c r="F12" s="4">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="G12" s="5">
-        <v>0.36</v>
+        <v>0.38</v>
       </c>
       <c r="K12">
         <v>4</v>
@@ -6449,13 +6449,13 @@
         <v>5</v>
       </c>
       <c r="L13" s="4">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="M13" s="4">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="N13" s="5">
-        <v>0.18518518518518517</v>
+        <v>0.2857142857142857</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
@@ -6478,10 +6478,10 @@
         <v>188</v>
       </c>
       <c r="M14" s="4">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="N14" s="5">
-        <v>0.31382978723404253</v>
+        <v>0.32978723404255317</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
@@ -6492,10 +6492,10 @@
         <v>188</v>
       </c>
       <c r="F15" s="4">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="G15" s="5">
-        <v>0.31382978723404253</v>
+        <v>0.32978723404255317</v>
       </c>
     </row>
   </sheetData>
@@ -14060,12 +14060,14 @@
         <v>1</v>
       </c>
       <c r="O136" s="12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P136" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q136" s="13"/>
+        <v>1</v>
+      </c>
+      <c r="Q136" s="13">
+        <v>46144</v>
+      </c>
       <c r="R136" s="12">
         <v>0</v>
       </c>
@@ -14133,7 +14135,7 @@
         <v>2026</v>
       </c>
       <c r="B138" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C138" s="1" t="s">
         <v>19</v>
@@ -14166,18 +14168,20 @@
         <v>191</v>
       </c>
       <c r="M138" s="13">
-        <v>45940</v>
+        <v>46065</v>
       </c>
       <c r="N138" s="12">
         <v>1</v>
       </c>
       <c r="O138" s="12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P138" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q138" s="13"/>
+        <v>1</v>
+      </c>
+      <c r="Q138" s="13">
+        <v>46161</v>
+      </c>
       <c r="R138" s="12">
         <v>0</v>
       </c>
@@ -14620,12 +14624,14 @@
         <v>1</v>
       </c>
       <c r="O146" s="12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P146" s="12">
-        <v>0</v>
-      </c>
-      <c r="Q146" s="13"/>
+        <v>1</v>
+      </c>
+      <c r="Q146" s="13">
+        <v>46158</v>
+      </c>
       <c r="R146" s="12">
         <v>0</v>
       </c>

</xml_diff>